<commit_message>
Rewrite BYOD remediation steps as admin console click paths
Every remediation and verification step now uses the Microsoft 365 admin
consoles (Microsoft 365, Entra, Intune, Exchange, SharePoint, Defender,
Purview) instead of PowerShell. Adds an Admin Consoles sheet with URLs
and least-privileged roles. The one setting with no console equivalent
(read-only OWA attachments) is called out with a Defender for Cloud Apps
alternative.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBuB8JFzWJ63ukfvtiahEJ
</commit_message>
<xml_diff>
--- a/byod/BYOD-Security-Remediation.xlsx
+++ b/byod/BYOD-Security-Remediation.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Remediation Plan" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Admin Consoles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Remediation Plan'!$A$1:$L$19</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -120,9 +126,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -155,6 +161,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -566,94 +578,118 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Columns to fill in</t>
+          <t>Admin consoles</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Owner and Status are for you to complete. Status values: Not started, In progress, Done, Accepted risk. Everything else is reference content.</t>
+          <t>All steps are written as click paths in the Microsoft 365 admin consoles (no PowerShell). The 'Admin Consoles' sheet lists each console's URL and the least-privileged admin role needed. Tip: every console has a search box at the top if a menu has moved.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Example</t>
+          <t>One exception</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Priority 2 &gt; Owner: J. Smith &gt; Status: In progress</t>
+          <t>Read-only Outlook on the web for unmanaged devices (item 4, step 5) has no admin-center switch; use a Defender for Cloud Apps session policy, or one Exchange PowerShell command if you do not have that licence.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Criticality</t>
+          <t>Columns to fill in</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Critical = exploitable now and leads to data loss or account takeover; High = significant exposure; Medium = gaps in governance or defence in depth; Low = residual risk.</t>
+          <t>Owner and Status are for you to complete. Status values: Not started, In progress, Done, Accepted risk. Everything else is reference content.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Licensing</t>
+          <t>Example</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Most controls need Microsoft Entra ID P1 and Intune, both in Microsoft 365 Business Premium (up to 300 users) and E3+EMS / E5. Risk-based policies need Entra ID P2.</t>
+          <t>Priority 2 &gt; Owner: J. Smith &gt; Status: In progress</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Recommended BYOD model</t>
+          <t>Criticality</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Phones/tablets: Intune app protection without enrolment (MAM). Personal Windows/macOS: browser-only or Edge with Windows MAM. Full desktop apps only on Intune-compliant devices.</t>
+          <t>Critical = exploitable now and leads to data loss or account takeover; High = significant exposure; Medium = gaps in governance or defence in depth; Low = residual risk.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>Licensing</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Introduce Conditional Access policies in Report-only mode first and always exclude two monitored break-glass admin accounts.</t>
+          <t>Most controls need Microsoft Entra ID P1 and Intune, both in Microsoft 365 Business Premium (up to 300 users) and E3+EMS / E5. Risk-based policies need Entra ID P2.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Recommended BYOD model</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Microsoft renames portal menus and retires controls regularly (e.g. 'Require approved client app'). Confirm against current Microsoft Learn documentation before changing production.</t>
+          <t>Phones/tablets: Intune app protection without enrolment (MAM). Personal Windows/macOS: browser-only or Edge with Windows MAM. Full desktop apps only on Intune-compliant devices.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Caution</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Introduce Conditional Access policies in Report-only mode first and always exclude two monitored break-glass admin accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft renames portal menus and retires controls regularly (e.g. 'Require approved client app'). Menu paths are current as of October 2026; confirm against Microsoft Learn before changing production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Prepared</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
@@ -678,10 +714,10 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="95" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
@@ -720,7 +756,7 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Where to configure</t>
+          <t>Admin console</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
@@ -775,15 +811,15 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>1. Inventory current licences: Microsoft 365 admin center &gt; Billing &gt; Your products.
-2. Move users who access company data from personal devices to Microsoft 365 Business Premium (up to 300 users) or E3 + EMS / E5.
-3. Decide whether you need Entra ID P2 (risk-based Conditional Access) and Defender for Cloud Apps (browser session control); both are in E5 or available as add-ons.
-4. Assign licences to all users before building the policies below; unlicensed users are not covered by Intune app protection.</t>
+          <t>1. Microsoft 365 admin center &gt; Billing &gt; Licenses: note which products you own and how many are assigned.
+2. Microsoft 365 admin center &gt; Users &gt; Active users &gt; Filter &gt; Unlicensed users: identify anyone without a licence.
+3. Microsoft 365 admin center &gt; Billing &gt; Purchase services: buy Microsoft 365 Business Premium (up to 300 users) or E3 + EMS E3 / E5. Add Entra ID P2 or Defender for Cloud Apps only if you want items 5 (risk policies) and 9 (browser session control).
+4. Microsoft 365 admin center &gt; Users &gt; Active users &gt; select users &gt; Manage product licenses &gt; Replace: assign the new licence to everyone who will use a personal device. Unlicensed users are not covered by Intune app protection.</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 admin center &gt; Billing; Users &gt; Active users &gt; Licenses</t>
+          <t>Microsoft 365 admin center (admin.microsoft.com) &gt; Billing; Users &gt; Active users</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
@@ -793,7 +829,7 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Get-MgSubscribedSku | Select SkuPartNumber, ConsumedUnits; confirm every active user has Entra ID P1 + Intune service plans.</t>
+          <t>Microsoft 365 admin center &gt; Billing &gt; Licenses shows Business Premium (or E3+EMS/E5) assigned to every active user; the Unlicensed users filter returns nobody who uses company data.</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
@@ -834,17 +870,18 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>1. If you have no Conditional Access licence, turn on Security Defaults (Entra admin center &gt; Identity &gt; Overview &gt; Properties).
-2. Otherwise create Conditional Access policies: 'Require MFA for all users' (all cloud apps) and 'Block legacy authentication' (Client apps = Exchange ActiveSync clients + Other clients).
-3. Start in Report-only mode for 1-2 weeks, review the sign-in logs, then switch to On.
-4. Exclude two cloud-only break-glass admin accounts, protected by FIDO2 keys and monitored.
-5. Move users to phishing-resistant methods (passkeys in Microsoft Authenticator, FIDO2 keys, Windows Hello) and use Authentication strengths to require them for admins.
-6. Disable POP/IMAP/SMTP AUTH where not needed: Set-CASMailbox -PopEnabled $false -ImapEnabled $false -SmtpClientAuthenticationDisabled $true (or via CAS mailbox plans).</t>
+          <t>1. No Conditional Access licence: Entra admin center &gt; Entra ID &gt; Overview &gt; Properties &gt; Manage security defaults &gt; Enabled. (Turn it off again once you build the policies below.)
+2. With Entra ID P1: Entra admin center &gt; Conditional Access &gt; Policies &gt; New policy from template &gt; 'Require multifactor authentication for all users' and 'Block legacy authentication'. Set each to Report-only.
+3. In each policy: Users &gt; Exclude &gt; add two cloud-only break-glass admin accounts.
+4. After 1-2 weeks, Entra admin center &gt; Sign-in logs &gt; filter Conditional Access = Report-only: failure to check who would be blocked, fix them, then set the policies to On.
+5. Entra admin center &gt; Authentication methods &gt; Policies: enable Passkey (FIDO2) and Microsoft Authenticator; then Conditional Access &gt; Authentication strengths &gt; use 'Phishing-resistant MFA' in a policy targeting admin roles.
+6. Exchange admin center &gt; Settings &gt; Mail flow &gt; tick 'Turn off SMTP AUTH protocol for your organization'.
+7. For users who do not need POP/IMAP: Microsoft 365 admin center &gt; Users &gt; Active users &gt; select user &gt; Mail &gt; Manage email apps &gt; untick POP, IMAP and Authenticated SMTP &gt; Save changes.</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Protection &gt; Conditional Access; Authentication methods; Exchange Online PowerShell</t>
+          <t>Entra admin center (entra.microsoft.com) &gt; Conditional Access, Authentication methods; Exchange admin center &gt; Settings; Microsoft 365 admin center &gt; Active users</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
@@ -854,7 +891,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Entra sign-in logs filtered on 'Client app = legacy' show only failures; Authentication methods &gt; User registration details shows 100% MFA-capable.</t>
+          <t>Entra admin center &gt; Sign-in logs &gt; filter Client app = the legacy client types: only failures appear. Entra admin center &gt; Authentication methods &gt; User registration details: every user is MFA capable.</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -895,17 +932,17 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>1. Decide the BYOD model per platform. Recommended: iOS/Android = app protection without enrolment (MAM); Windows/macOS personal = browser-only or Edge with Windows MAM; full desktop apps only on Intune-compliant devices.
-2. Create a CA policy for iOS/Android: grant 'Require app protection policy' (the older 'Require approved client app' control is being retired).
-3. Create a CA policy for Windows/macOS desktop clients: 'Require device to be marked as compliant' (Client apps = Mobile apps and desktop clients).
-4. Create a CA policy for browsers on unmanaged devices: Session &gt; 'Use app enforced restrictions' (pairs with item 4 below).
-5. Block unsupported device platforms (e.g. Linux, unknown) unless there is a business need.
-6. Pilot with a test group in Report-only, then enforce.</t>
+          <t>Decide the model first: phones/tablets = app protection without enrolment; personal Windows/Mac = browser only (or Edge with Windows MAM); full desktop apps only on Intune-compliant devices.
+1. Entra admin center &gt; Conditional Access &gt; Policies &gt; New policy 'BYOD - mobile apps need app protection': Users = All users (exclude break-glass); Target resources = Office 365; Conditions &gt; Device platforms = iOS, Android; Grant = 'Require app protection policy'. (The older 'Require approved client app' control is being retired.)
+2. New policy 'Desktop apps need compliant device': Device platforms = Windows, macOS; Conditions &gt; Client apps = Mobile apps and desktop clients; Grant = 'Require device to be marked as compliant'.
+3. New policy 'Browser on unmanaged devices': Client apps = Browser; Session = 'Use app enforced restrictions' (works with the SharePoint/Outlook settings in item 4).
+4. New policy 'Block unknown platforms': Device platforms &gt; Include Any device &gt; Exclude Android, iOS, Windows, macOS; Grant = Block access.
+5. Create every policy as Report-only, test with Conditional Access &gt; Policies &gt; What If, then switch to On.</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Protection &gt; Conditional Access</t>
+          <t>Entra admin center (entra.microsoft.com) &gt; Conditional Access &gt; Policies</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -915,7 +952,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Use the Conditional Access 'What If' tool for a user on an unregistered iPhone and an unmanaged Windows PC; check sign-in logs show the expected grant control.</t>
+          <t>Entra admin center &gt; Conditional Access &gt; What If: a user on iOS gets 'Require app protection policy', on an unmanaged Windows desktop client gets 'Require compliant device'. Sign-in logs &gt; Conditional Access tab shows the expected policy applied.</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -956,28 +993,28 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>1. In Intune create App protection policies for iOS and Android targeting all users and core apps (Outlook, Teams, OneDrive, SharePoint, Word/Excel/PowerPoint, Edge). Start from the Microsoft 'Level 2 enhanced data protection' framework.
-2. Data settings: block backup to iCloud/Google, 'Send org data to other apps' = Policy managed apps, 'Save copies of org data' = Block (allow OneDrive/SharePoint only), restrict cut/copy/paste to policy-managed apps, encrypt org data, block screen capture (Android).
-3. Access settings: require app PIN or biometrics, re-check after 30 minutes of inactivity.
-4. SharePoint/OneDrive on unmanaged devices: Set-SPOTenant -ConditionalAccessPolicy AllowLimitedAccess (web view only, no download/print/sync).
-5. Outlook on the web on unmanaged devices: Set-OwaMailboxPolicy -Identity OwaMailboxPolicy-Default -ConditionalAccessPolicy ReadOnly (attachments viewable, not downloadable).
-6. Windows personal PCs: enable Intune 'Windows MAM' for Microsoft Edge so the browser is the protected container.
-7. Note: the OneDrive 'sync only on domain-joined PCs' setting needs on-premises AD and does not apply to a cloud-only tenant; use the compliant-device CA policy (item 3) to control sync.</t>
+          <t>1. Intune admin center &gt; Apps &gt; App protection policies &gt; Create policy &gt; iOS/iPadOS (repeat for Android). Apps: Target to 'All Microsoft apps' (or select Outlook, Teams, OneDrive, SharePoint, Word, Excel, PowerPoint, Edge). Assignments: All users.
+2. Data protection page: Backup org data to iTunes/iCloud/Google = Block; Send org data to other apps = Policy managed apps; Save copies of org data = Block, Allow user to save copies to = OneDrive for Business, SharePoint; Restrict cut, copy and paste = Policy managed apps with paste in; Encrypt org data = Require; Screen capture (Android) = Block.
+3. Access requirements page: PIN for access = Require (biometrics allowed); Recheck after (minutes of inactivity) = 30.
+4. SharePoint admin center &gt; Policies &gt; Access control &gt; Unmanaged devices &gt; 'Allow limited, web-only access' &gt; Save. (This also creates matching Conditional Access policies in Entra; review them there.)
+5. Outlook on the web: Exchange has no admin-center switch for read-only attachments. Use Defender portal &gt; Cloud apps &gt; Policies &gt; Policy management &gt; Create policy &gt; Session policy &gt; 'Block download based on real-time content inspection' scoped to unmanaged devices (needs Defender for Cloud Apps). Without that licence, the only option is one Exchange PowerShell command (Set-OwaMailboxPolicy ... -ConditionalAccessPolicy ReadOnly).
+6. Personal Windows PCs: Intune admin center &gt; Apps &gt; App protection policies &gt; Create policy &gt; Windows (Microsoft Edge), then in Entra a CA policy for Windows + Browser with Grant 'Require app protection policy'.
+7. The OneDrive 'sync only on domain-joined PCs' setting needs on-premises AD and does not apply to a cloud-only tenant; the compliant-device policy in item 3 controls sync instead.</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Intune admin center &gt; Apps &gt; App protection policies; SharePoint Online PowerShell; Exchange Online PowerShell</t>
+          <t>Intune admin center (intune.microsoft.com) &gt; Apps &gt; App protection policies; SharePoint admin center &gt; Policies &gt; Access control; Defender portal &gt; Cloud apps</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Intune + Entra ID P1</t>
+          <t>Intune + Entra ID P1 (Defender for Cloud Apps for step 5)</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>On a test personal phone, try to 'Save to Files' an Outlook attachment and paste mail text into a personal app (both blocked); open SharePoint in a browser on an unmanaged PC (download button absent).</t>
+          <t>On a test personal phone, 'Save to Files' from Outlook and pasting mail text into a personal app are both blocked. In a browser on an unmanaged PC, SharePoint shows the 'download disabled' banner. Intune admin center &gt; Apps &gt; Monitor &gt; App protection status lists the test user.</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -1018,17 +1055,17 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>1. Require phishing-resistant MFA (passkeys / FIDO2) where possible; it defeats AiTM proxies.
-2. For unmanaged devices set Session controls: Sign-in frequency (e.g. 8-12 hours) and 'Persistent browser session' = Never persistent.
-3. Turn on Continuous Access Evaluation and, if you use named locations, strict location enforcement.
-4. Where supported, enable Token protection (CA session control) for Exchange/SharePoint/Teams on Windows; check current platform support before relying on it.
-5. With Entra ID P2, add risk-based policies: sign-in risk High/Medium = MFA, user risk High = secure password change.
-6. Prepare a response playbook: Revoke-MgUserSignInSession -UserId &lt;user&gt;, reset password, review inbox rules and forwarding (Get-InboxRule), and check audit logs.</t>
+          <t>1. Entra admin center &gt; Authentication methods &gt; Policies: enable Passkey (FIDO2) and roll out passkeys in Microsoft Authenticator; phishing-resistant methods defeat AiTM proxies.
+2. Entra admin center &gt; Conditional Access &gt; New policy 'Unmanaged device sessions': Conditions &gt; Filter for devices &gt; exclude compliant devices (device.isCompliant -eq True); Session &gt; Sign-in frequency = 8 hours and Persistent browser session = Never persistent.
+3. In the same policy, Session &gt; Customize continuous access evaluation: leave enabled; if you use named locations choose 'Strictly enforce location policies'.
+4. Where your platforms support it, Session &gt; 'Require token protection for sign-in sessions' for Exchange Online, SharePoint and Teams (check Microsoft's current platform list first).
+5. With Entra ID P2: new CA policies using Conditions &gt; Sign-in risk (High, Medium) = Require MFA, and Conditions &gt; User risk (High) = Require password change.
+6. Compromise playbook in the consoles: Microsoft 365 admin center &gt; Active users &gt; user &gt; Account &gt; 'Sign out of all sessions' (or Entra admin center &gt; Users &gt; user &gt; Revoke sessions); Reset password; Exchange admin center &gt; Mailboxes &gt; user &gt; Mail flow settings &gt; check Email forwarding; Purview portal &gt; Audit &gt; search activities 'New-InboxRule' / 'Set-InboxRule' for that user; Exchange admin center &gt; Reports &gt; Mail flow &gt; Auto forwarded messages.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Conditional Access; Entra ID Protection; Microsoft Graph PowerShell</t>
+          <t>Entra admin center &gt; Conditional Access, Authentication methods, Users; Microsoft 365 admin center; Exchange admin center; Purview portal &gt; Audit</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -1038,7 +1075,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Sign-in logs show sign-in frequency enforced for unmanaged devices; run the playbook against a test account and confirm sessions end within minutes.</t>
+          <t>Entra admin center &gt; Sign-in logs &gt; a sign-in from an unmanaged device shows sign-in frequency applied. Run the playbook on a test account: the user is signed out of Outlook/Teams within minutes.</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1080,15 +1117,16 @@
       <c r="F7" s="7" t="inlineStr">
         <is>
           <t>1. Rely on app protection (item 4) so corporate data lives only inside managed apps.
-2. Set conditional launch 'Offline grace period' to wipe data after e.g. 90 days without check-in.
-3. Add to the leaver and lost-device process: Intune &gt; Apps &gt; App selective wipe; disable the account; Revoke-MgUserSignInSession.
-4. For native mail apps that are still allowed: Clear-MobileDevice -Identity &lt;id&gt; -AccountOnly (Exchange account-only wipe, leaves personal data).
-5. Tell users how to report a lost device within hours, not days.</t>
+2. Intune admin center &gt; Apps &gt; App protection policies &gt; open each policy &gt; Properties &gt; Conditional launch &gt; Edit: Offline grace period = Wipe data after 90 days.
+3. Lost device or leaver: Intune admin center &gt; Apps &gt; App selective wipe &gt; Create wipe request &gt; choose the user and device.
+4. Microsoft 365 admin center &gt; Active users &gt; user &gt; Block sign-in, then Account &gt; 'Sign out of all sessions'.
+5. If native mail apps are still allowed: Exchange admin center &gt; Recipients &gt; Mailboxes &gt; select user &gt; Others &gt; Manage mobile devices &gt; select the device &gt; 'Account only remote wipe device' (removes the mailbox only, leaves personal data).
+6. Add these steps to the HR leaver checklist and tell users to report a lost device within hours.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Intune admin center &gt; Apps &gt; App selective wipe; Exchange Online PowerShell; HR offboarding procedure</t>
+          <t>Intune admin center &gt; Apps &gt; App selective wipe; Microsoft 365 admin center &gt; Active users; Exchange admin center &gt; Mailboxes</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1098,7 +1136,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Run a selective wipe against a test phone: corporate accounts and files disappear from Outlook/OneDrive/Teams, personal photos and apps remain.</t>
+          <t>Create a selective wipe for a test phone: Intune admin center &gt; Apps &gt; App selective wipe shows status Done; company accounts and files disappear from Outlook/OneDrive/Teams while personal photos and apps remain.</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -1139,15 +1177,15 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>1. In app protection policies set Conditional launch: minimum OS version (block or wipe below it), jailbroken/rooted = Block access, Play Integrity verdict = Basic integrity and certified device (Android), minimum app versions.
-2. Optionally connect Microsoft Defender for Endpoint on iOS/Android and set 'Max allowed device threat level' in conditional launch.
-3. For personal devices you do enrol (iOS/iPadOS User Enrollment, Android Work Profile), create compliance policies with minimum OS, passcode and encryption requirements.
-4. Set Intune compliance 'Mark devices with no compliance policy assigned as' = Not compliant.</t>
+          <t>1. Intune admin center &gt; Apps &gt; App protection policies &gt; open each policy &gt; Properties &gt; Conditional launch &gt; Edit. Device conditions: Jailbroken/rooted devices = Block access; Min OS version = current major minus one, action Block access; Play integrity verdict (Android) = Basic integrity &amp; device certification, Block access. App conditions: Min app version where needed.
+2. Optional mobile threat defence: Intune admin center &gt; Endpoint security &gt; Microsoft Defender for Endpoint &gt; turn on 'Connect Android/iOS devices to Microsoft Defender for Endpoint' for app protection policy evaluation; then in Conditional launch add Max allowed device threat level = Low.
+3. For personal devices you enrol (iOS User Enrollment, Android Work Profile): Intune admin center &gt; Devices &gt; Compliance &gt; Create policy: minimum OS, require passcode and encryption.
+4. Intune admin center &gt; Devices &gt; Compliance &gt; Compliance settings: 'Mark devices with no compliance policy assigned as' = Not compliant.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Intune admin center &gt; Apps &gt; App protection policies &gt; Conditional launch; Devices &gt; Compliance</t>
+          <t>Intune admin center (intune.microsoft.com) &gt; Apps &gt; App protection policies; Devices &gt; Compliance; Endpoint security</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -1157,7 +1195,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Intune &gt; Apps &gt; Monitor &gt; App protection status shows no users on blocked OS versions; test with an old OS emulator or device.</t>
+          <t>Intune admin center &gt; Apps &gt; Monitor &gt; App protection status &gt; App protection report: no users on blocked OS versions. A test device below the minimum OS is blocked on launch.</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -1198,15 +1236,16 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>1. Standardise on Outlook for iOS/Android and communicate the change in advance.
-2. Conditional Access: block 'Exchange ActiveSync clients' (or require app protection, which native apps cannot satisfy).
-3. Defence in depth: Set-ActiveSyncOrganizationSettings -DefaultAccessLevel Quarantine and approve only Outlook via device access rules, or disable ActiveSync for users who do not need it (Set-CASMailbox -ActiveSyncEnabled $false).
-4. Review which devices already sync: Get-MobileDevice -ResultSize Unlimited | Group DeviceOS, ClientType.</t>
+          <t>1. See who uses what: Microsoft 365 admin center &gt; Reports &gt; Usage &gt; Exchange &gt; Email apps usage.
+2. Announce the move to Outlook for iOS/Android, with a date.
+3. Entra admin center &gt; Conditional Access &gt; New policy 'Block ActiveSync': Conditions &gt; Client apps &gt; Exchange ActiveSync clients; Target resources = Office 365 Exchange Online; Grant = Block access. Report-only first, then On.
+4. Defence in depth: Exchange admin center &gt; Mobile &gt; Device access &gt; Edit: when a device that is not managed by a rule connects = Quarantine; then add a device access rule allowing Outlook.
+5. Users who need no mobile mail at all: Microsoft 365 admin center &gt; Active users &gt; user &gt; Mail &gt; Manage email apps &gt; untick Exchange ActiveSync.</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Conditional Access; Exchange admin center &gt; Mobile; Exchange Online PowerShell</t>
+          <t>Entra admin center &gt; Conditional Access; Exchange admin center &gt; Mobile &gt; Device access; Microsoft 365 admin center &gt; Reports</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -1216,7 +1255,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Adding the work account to iOS Mail fails; Get-MobileDevice shows only Outlook (ClientType REST/Outlook) after cleanup.</t>
+          <t>Adding the work account to iOS Mail fails. Microsoft 365 admin center &gt; Reports &gt; Usage &gt; Email apps usage shows Outlook for mobile only after cleanup.</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1257,16 +1296,16 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>1. Block desktop/mobile clients on non-compliant Windows/macOS (item 3, policy for desktop clients).
-2. Allow browser access with app-enforced restrictions (SharePoint limited access, OWA ReadOnly - see item 4).
-3. Preferably require Microsoft Edge with Windows MAM on personal Windows PCs (CA: Windows platform, browser, grant 'Require app protection policy').
-4. With Defender for Cloud Apps, use Conditional Access App Control session policies to block download / copy / print of sensitive content in any browser.
-5. Educate users that personal PCs are browser-only by design.</t>
+          <t>1. Desktop apps blocked on non-compliant Windows/macOS: the 'Desktop apps need compliant device' policy from item 3.
+2. Browser access limited: the SharePoint 'Allow limited, web-only access' setting and the browser policy from items 3-4.
+3. Preferred on personal Windows: Intune admin center &gt; Apps &gt; App protection policies &gt; Create policy &gt; Windows (Microsoft Edge) with Data protection &gt; Receive data from / Send data to = Org data sources only, Print org data = Block. Then Entra admin center &gt; Conditional Access &gt; New policy: Device platforms = Windows, Client apps = Browser, Grant = Require app protection policy. Users get the Edge work profile.
+4. With Defender for Cloud Apps: Defender portal &gt; Cloud apps &gt; Policies &gt; Policy management &gt; Create policy &gt; Session policy: Session control type = Control file download (with inspection), Activity source = device tag not Intune compliant, Action = Block (also add policies for print and copy/paste as needed).
+5. Explain to users that personal PCs are browser-only by design.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Conditional Access; Intune &gt; App protection (Windows); Defender portal &gt; Cloud apps</t>
+          <t>Entra admin center &gt; Conditional Access; Intune admin center &gt; App protection policies (Windows); Defender portal (security.microsoft.com) &gt; Cloud apps</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1276,7 +1315,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>On a personal PC: Outlook desktop sign-in blocked, OWA attachments are view-only, SharePoint shows 'download disabled' banner.</t>
+          <t>On a personal PC: Outlook desktop sign-in is blocked, SharePoint shows the 'download disabled' banner, and (with Cloud Apps) a download attempt shows the block page. Defender portal &gt; Cloud apps &gt; Activity log records it.</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -1317,15 +1356,15 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>1. Entra admin center &gt; Devices &gt; Device settings: limit 'Maximum number of devices per user' (e.g. 5-10).
-2. Create a CA policy for the user action 'Register or join devices' requiring MFA (set 'Require MFA to register or join devices' to No when using the CA policy).
-3. Intune &gt; Devices &gt; Enrollment restrictions: block personally owned Windows/macOS enrolment if the BYOD model is MAM-only; allow iOS User Enrollment / Android Work Profile only.
-4. Schedule clean-up of devices inactive for 90+ days (Entra &gt; Devices &gt; All devices, filter Activity), disable first and delete after a grace period.</t>
+          <t>1. Entra admin center &gt; Devices &gt; Device settings: Maximum number of devices per user = 10 (or fewer).
+2. Entra admin center &gt; Conditional Access &gt; New policy: Target resources &gt; User actions &gt; 'Register or join devices'; Grant = Require multifactor authentication. Then in Devices &gt; Device settings set 'Require Multifactor Authentication to register or join devices' = No (the CA policy replaces it).
+3. Intune admin center &gt; Devices &gt; Enrollment &gt; Device platform restriction &gt; edit the default Windows and macOS restrictions: Personally owned devices = Block (if personal PCs are browser only). For iOS allow User Enrollment; for Android allow Work Profile only.
+4. Monthly: Entra admin center &gt; Devices &gt; All devices &gt; Columns: Activity &gt; filter devices inactive 90+ days &gt; Disable; delete after a further grace period.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Devices &gt; Device settings; Conditional Access; Intune &gt; Enrollment</t>
+          <t>Entra admin center &gt; Devices &gt; Device settings, All devices; Conditional Access; Intune admin center &gt; Devices &gt; Enrollment</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1335,7 +1374,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Registering a new device prompts for MFA; Intune enrollment of a personal Windows PC is blocked; stale-device report is reviewed monthly.</t>
+          <t>Registering a new device prompts for MFA. Enrolling a personal Windows PC into Intune is refused. Entra admin center &gt; Devices &gt; All devices shows no active devices older than 90 days.</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -1376,15 +1415,15 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>1. Entra admin center &gt; Enterprise apps &gt; Consent and permissions: allow user consent only for apps from verified publishers with low-impact permissions (or disable user consent).
-2. Enable the admin consent workflow so users can request apps and admins review them.
-3. Review existing grants: Enterprise apps &gt; filter 'Application type = all', check permissions and remove unknown apps.
-4. With Defender for Cloud Apps, enable app governance / OAuth app policies to alert on risky apps.</t>
+          <t>1. Entra admin center &gt; Enterprise apps &gt; Consent and permissions &gt; User consent settings: 'Allow user consent for apps from verified publishers, for selected permissions' (or 'Do not allow user consent').
+2. Same page &gt; Admin consent settings: Users can request admin consent = Yes; choose reviewers.
+3. Entra admin center &gt; Enterprise apps &gt; All applications &gt; Application type = All applications: open each unfamiliar app &gt; Permissions; remove apps you do not recognise (Properties &gt; Delete).
+4. With Defender for Cloud Apps: Defender portal &gt; Cloud apps &gt; App governance: turn on and review the predefined OAuth app policies.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Enterprise applications &gt; Consent and permissions</t>
+          <t>Entra admin center &gt; Enterprise apps &gt; Consent and permissions; Defender portal &gt; Cloud apps &gt; App governance</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1394,7 +1433,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>A test user attempting to consent to an unverified app with Mail.Read sees 'Approval required'.</t>
+          <t>A test user who tries to consent to an unverified app requesting Mail.Read sees 'Approval required'. Entra admin center &gt; Enterprise apps &gt; Admin consent requests receives the request.</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -1435,16 +1474,16 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>1. Confirm the unified audit log is on: Get-AdminAuditLogConfig | fl UnifiedAuditLogIngestionEnabled.
-2. Export Entra sign-in and audit logs to a Log Analytics workspace or SIEM for 90+ days of retention.
-3. Use the Conditional Access insights and reporting workbook to see unmanaged-device sign-ins.
-4. Review Intune app protection reports monthly (Apps &gt; Monitor &gt; App protection status).
-5. Create alerts for new inbox forwarding rules, mass downloads and impossible travel (Defender portal alert policies).</t>
+          <t>1. Microsoft Purview portal &gt; Solutions &gt; Audit: if a banner says 'Start recording user and admin activity', select it (auditing is on by default in most tenants).
+2. Entra admin center &gt; Monitoring &amp; health &gt; Diagnostic settings &gt; Add diagnostic setting: send SignInLogs, NonInteractiveUserSignInLogs and AuditLogs to a Log Analytics workspace (Azure subscription) with 90+ days retention.
+3. Entra admin center &gt; Monitoring &amp; health &gt; Workbooks &gt; 'Conditional Access insights and reporting': review unmanaged-device sign-ins monthly.
+4. Intune admin center &gt; Apps &gt; Monitor &gt; App protection status: review monthly.
+5. Defender portal &gt; Email &amp; collaboration &gt; Policies &amp; rules &gt; Alert policy: make sure alerts for 'Suspicious email forwarding activity' and 'Creation of forwarding/redirect rule' are on and notify an admin mailbox.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Monitoring &gt; Diagnostic settings; Purview portal &gt; Audit; Defender portal</t>
+          <t>Purview portal (purview.microsoft.com) &gt; Audit; Entra admin center &gt; Monitoring &amp; health; Defender portal &gt; Policies &amp; rules</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -1454,7 +1493,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>A sign-in from a test unmanaged device can be found in the SIEM 60 days later.</t>
+          <t>Purview &gt; Audit search returns events from today. A sign-in from a test unmanaged device can still be found in Log Analytics 60 days later.</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
@@ -1495,15 +1534,15 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>1. Create a small label taxonomy (Public, General, Confidential, Highly Confidential) in Microsoft Purview.
-2. Apply encryption to Confidential and above so files can only be opened by authorised users, and optionally block offline access for Highly Confidential.
-3. Configure DLP policies for Exchange, SharePoint, OneDrive and Teams to detect and block sharing of sensitive information types (payment cards, national IDs).
-4. Turn on default labelling for new documents and mail where appropriate.</t>
+          <t>1. Microsoft Purview portal &gt; Solutions &gt; Information protection &gt; Sensitivity labels &gt; Create a label: Public, General, Confidential, Highly Confidential.
+2. For Confidential and Highly Confidential: Items &gt; Control access (encryption) &gt; assign permissions to your organisation; for Highly Confidential set 'Allow offline access' = Never.
+3. Information protection &gt; Label publishing policies &gt; Publish labels to all users; optionally set a default label.
+4. Purview portal &gt; Solutions &gt; Data loss prevention &gt; Policies &gt; Create policy: use a template (e.g. Financial / Privacy for your country), locations Exchange, SharePoint, OneDrive, Teams, action Block sharing outside the organisation with policy tips. Start in simulation mode.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Microsoft Purview portal &gt; Information protection; Data loss prevention</t>
+          <t>Microsoft Purview portal (purview.microsoft.com) &gt; Information protection; Data loss prevention</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1513,7 +1552,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Open a Highly Confidential document as an unauthorised user (denied); DLP blocks emailing a test card number externally.</t>
+          <t>An unauthorised user cannot open a Highly Confidential test file. Emailing a test credit-card number externally triggers the DLP policy tip and appears under Purview &gt; Data loss prevention &gt; Alerts.</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
@@ -1554,16 +1593,16 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>1. Write a BYOD policy with HR and legal: eligible devices, required apps (Outlook, Teams, OneDrive), minimum OS, PIN/biometric, reporting loss within 24 hours, selective-wipe consent, what IT can and cannot see.
-2. Prefer MAM or user enrolment models so IT never sees personal apps, photos or location.
-3. Customise Intune Company Portal privacy messaging and terms and conditions.
-4. Require acknowledgement (Entra terms of use, enforceable via Conditional Access) before access.
-5. Review the policy annually.</t>
+          <t>1. Write the policy with HR and legal: eligible devices, required apps, minimum OS, PIN/biometric, report loss within 24 hours, consent to selective wipe, what IT can and cannot see.
+2. Entra admin center &gt; Conditional Access &gt; Terms of use &gt; New terms: upload the policy PDF, Require users to expand = On.
+3. Entra admin center &gt; Conditional Access &gt; New policy 'Accept BYOD terms': All users, Office 365, Grant = the terms of use you created.
+4. Intune admin center &gt; Tenant administration &gt; Customization &gt; edit: add privacy statement URL, support contact and the Company Portal message explaining what IT can see.
+5. Review the policy every year and publish a new terms-of-use version when it changes.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>HR/legal; Entra admin center &gt; Identity governance &gt; Terms of use; Intune &gt; Tenant administration &gt; Customization</t>
+          <t>Entra admin center &gt; Conditional Access &gt; Terms of use; Intune admin center &gt; Tenant administration &gt; Customization</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1573,7 +1612,7 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Every BYOD user has accepted the current terms of use version (Terms of use report).</t>
+          <t>Entra admin center &gt; Conditional Access &gt; Terms of use &gt; select the terms &gt; View accepted/declined shows every BYOD user accepted the current version.</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1614,15 +1653,15 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>1. Rely on app protection 'multi-identity' behaviour: org data cannot be saved to the personal account inside Outlook/OneDrive/Office (item 4 settings).
-2. Use Edge for Business profiles; on Windows MAM the work profile is the protected container.
-3. Configure Entra Tenant restrictions v2 to stop users signing in to other tenants on devices where it can be enforced (managed devices or via Global Secure Access).
-4. Restrict external sharing in SharePoint/OneDrive to existing guests or specific domains.</t>
+          <t>1. App protection (item 4) already separates accounts inside Outlook/OneDrive/Office: confirm 'Save copies of org data' = Block with only OneDrive for Business and SharePoint allowed.
+2. Personal Windows: the Edge work profile created by Windows MAM (item 9) keeps work browsing separate.
+3. Entra admin center &gt; External Identities &gt; Cross-tenant access settings &gt; Default settings &gt; Tenant restrictions: block access to other tenants for your users. Note it is only enforced on managed devices or through Global Secure Access, not on unmanaged personal devices.
+4. SharePoint admin center &gt; Policies &gt; Sharing: set external sharing to 'Existing guests' or 'New and existing guests' and limit by domain (More external sharing settings).</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Intune &gt; App protection; Entra admin center &gt; External identities &gt; Cross-tenant access; SharePoint admin center &gt; Sharing</t>
+          <t>Intune admin center &gt; App protection policies; Entra admin center &gt; External Identities; SharePoint admin center &gt; Policies &gt; Sharing</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
@@ -1632,7 +1671,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>On a test phone, try to save a work attachment to the personal OneDrive account in the same app (blocked).</t>
+          <t>On a test phone, saving a work attachment to the personal OneDrive account in the same app is blocked.</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -1673,15 +1712,15 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>1. Run short onboarding training: installing Outlook/Teams, what app protection does, how to report loss or suspected compromise.
-2. Use Defender for Office 365 Attack simulation training (Plan 2) or another phishing simulator.
-3. Enable the Report Message / Report Phishing button in Outlook.
-4. Publish a one-page 'lost device' procedure with the helpdesk contact.</t>
+          <t>1. Run short onboarding training: installing Outlook/Teams from the official stores, what app protection does, how to report loss or compromise.
+2. Defender portal &gt; Email &amp; collaboration &gt; Attack simulation training &gt; Simulations &gt; Launch a simulation (Defender for Office 365 Plan 2).
+3. Defender portal &gt; Settings &gt; Email &amp; collaboration &gt; User reported settings: enable the Microsoft Report button in Outlook and set a reporting mailbox.
+4. Publish a one-page 'lost device' procedure with the helpdesk contact; link it in the Company Portal (Intune admin center &gt; Tenant administration &gt; Customization).</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Defender portal &gt; Email &amp; collaboration &gt; Attack simulation training; internal comms</t>
+          <t>Defender portal (security.microsoft.com) &gt; Attack simulation training; Settings &gt; Email &amp; collaboration</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1691,7 +1730,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Training completion rate and simulated phish click rate tracked quarterly.</t>
+          <t>Defender portal &gt; Attack simulation training &gt; Reports: completion and click rates tracked quarterly. Reported messages appear under Actions &amp; submissions &gt; Submissions.</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
@@ -1732,14 +1771,15 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>1. Define named locations for countries you operate in and block or require stronger MFA from others (do not rely on IP alone).
-2. Keep MFA and token controls (items 2 and 5) as the primary protection.
-3. Optionally evaluate Microsoft Entra Internet Access / Global Secure Access for compliant-network checks.</t>
+          <t>1. Entra admin center &gt; Conditional Access &gt; Named locations &gt; + Countries location: add the countries you operate in.
+2. Conditional Access &gt; New policy: Conditions &gt; Locations &gt; Include Any location, Exclude your countries location; Grant = Block access (or require phishing-resistant MFA). Exclude break-glass accounts and remember travelling staff.
+3. Keep MFA and session controls (items 2 and 5) as the main protection.
+4. Optional: Entra admin center &gt; Global Secure Access to add compliant-network checks.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Entra admin center &gt; Conditional Access &gt; Named locations</t>
+          <t>Entra admin center &gt; Conditional Access &gt; Named locations, Policies</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -1749,7 +1789,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>A test sign-in through a VPN exit node in a blocked country is denied.</t>
+          <t>Conditional Access &gt; What If with a blocked country selected returns Block access; sign-in logs show the policy blocking a test sign-in through a foreign VPN.</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
@@ -1791,9 +1831,9 @@
       <c r="F19" s="7" t="inlineStr">
         <is>
           <t>1. Prefer blocking sync on unmanaged PCs (items 3 and 4) so this cannot occur.
-2. Know the recovery tools: OneDrive 'Restore your OneDrive' (30 days), recycle bins (93 days).
-3. Apply Purview retention policies to Exchange, SharePoint and OneDrive for business-critical data.
-4. Consider Microsoft 365 Backup or a third-party backup for longer recovery points.</t>
+2. Know the recovery paths: user's OneDrive &gt; Settings &gt; Restore your OneDrive (30 days); SharePoint site &gt; Recycle bin (93 days).
+3. Microsoft Purview portal &gt; Solutions &gt; Data lifecycle management &gt; Policies &gt; Retention policies &gt; New retention policy: Exchange mailboxes, SharePoint sites, OneDrive accounts; retain for the period your business needs.
+4. Microsoft 365 admin center &gt; Settings &gt; Microsoft 365 Backup: set up billing and backup policies for critical OneDrive accounts, SharePoint sites and mailboxes.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1808,7 +1848,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>Test-restore a deleted folder from a pilot user's OneDrive.</t>
+          <t>Restore a deleted test folder from a pilot user's OneDrive; Purview &gt; Data lifecycle management &gt; Retention policies shows the policy On for all three locations.</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -1969,4 +2009,200 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Console</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Least-privileged role</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft 365 admin center</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>https://admin.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Licences, users, email apps per user, sign out of sessions, usage reports, Microsoft 365 Backup</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Global Reader to view; User Administrator / Billing Administrator to change</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft Entra admin center</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>https://entra.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Conditional Access, authentication methods, device settings, enterprise app consent, terms of use, sign-in logs</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Conditional Access Administrator, Authentication Policy Administrator, Cloud Application Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft Intune admin center</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>https://intune.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>App protection policies, selective wipe, compliance, enrolment restrictions, Company Portal customisation</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Intune Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Exchange admin center</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>https://admin.exchange.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>SMTP AUTH, mobile device access, mailbox forwarding, account-only wipe, mail flow reports</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>Exchange Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>SharePoint admin center</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>https://&lt;tenant&gt;-admin.sharepoint.com (or Microsoft 365 admin center &gt; Admin centers &gt; SharePoint)</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Unmanaged device access, external sharing</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>SharePoint Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft Defender portal</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>https://security.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Cloud Apps session policies and app governance, alert policies, attack simulation, user-reported settings</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Security Administrator</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Microsoft Purview portal</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>https://purview.microsoft.com</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Audit, sensitivity labels, DLP, retention</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Compliance Administrator</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>